<commit_message>
end of the chapter
</commit_message>
<xml_diff>
--- a/learn-english.xlsx
+++ b/learn-english.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/andreadipaola/Documents/GitHub/responsive-design/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{41E6CAF5-B5D2-0D4B-86C2-A61464AC02FF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E61937F2-A8EE-BE40-9F5E-779C0A26D870}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="14080" yWindow="1600" windowWidth="14720" windowHeight="16260" xr2:uid="{7364E0F6-D0AA-D842-BE53-618D0A6AFC46}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="52">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="54">
   <si>
     <t>English</t>
   </si>
@@ -181,6 +181,12 @@
   </si>
   <si>
     <t>non sarebbe fanstastico</t>
+  </si>
+  <si>
+    <t>scuffles back</t>
+  </si>
+  <si>
+    <t>rimoscolano</t>
   </si>
 </sst>
 </file>
@@ -580,7 +586,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C8F3ACB1-4208-5A47-A40E-2A91A8F2B8B9}">
-  <dimension ref="A1:B26"/>
+  <dimension ref="A1:B27"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="70.1640625" customWidth="1"/>
@@ -795,6 +801,14 @@
         <v>51</v>
       </c>
     </row>
+    <row r="27" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A27" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="B27" t="s">
+        <v>53</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>